<commit_message>
fix(grid): prioritize 独立屋销控表 tab as default active tab and naturally sort towers in app.js and Excel workbooks
</commit_message>
<xml_diff>
--- a/files/九龙-九龙塘-博峰.xlsx
+++ b/files/九龙-九龙塘-博峰.xlsx
@@ -8,9 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="销控汇总明细" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="住宅大楼 - 东翼" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="住宅大楼 - 西翼" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="独立屋销控表" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="独立屋销控表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="住宅大楼 - 东翼" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="住宅大楼 - 西翼" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4001,23 +4001,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>住宅大楼 - 东翼 销控网格图</t>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>博峰 - 独立屋销控网格图</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>总套数</t>
         </is>
@@ -4048,320 +4048,83 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C3" s="14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E3" s="16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F3" s="17" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
-        <is>
-          <t>楼层</t>
-        </is>
-      </c>
-      <c r="B4" s="18" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C4" s="18" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>A | 2217呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C5" s="20" t="inlineStr"/>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>12</t>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>2 套</t>
+        </is>
+      </c>
+      <c r="B3" s="22" t="inlineStr">
+        <is>
+          <t>0 套</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>0 套</t>
+        </is>
+      </c>
+      <c r="D3" s="24" t="inlineStr">
+        <is>
+          <t>0 套</t>
+        </is>
+      </c>
+      <c r="E3" s="25" t="inlineStr">
+        <is>
+          <t>0 套</t>
+        </is>
+      </c>
+      <c r="F3" s="21" t="inlineStr">
+        <is>
+          <t>2 套</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>类型/位置</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>1号屋</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2号屋</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>独立屋</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>A | 2207呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C6" s="20" t="inlineStr"/>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C7" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="58" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="58" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="58" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B13" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C13" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="58" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="58" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C15" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="58" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
+          <t>1号屋
+2623呎 (4+房)
+(待售)
+暂无价格
+暂无呎价</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>2号屋
+2621呎 (4+房)
+(待售)
+暂无价格
+暂无呎价</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
@@ -4385,7 +4148,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>住宅大楼 - 西翼 销控网格图</t>
+          <t>住宅大楼 - 东翼 销控网格图</t>
         </is>
       </c>
     </row>
@@ -4494,7 +4257,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>A | 2207呎 (4+房)
+          <t>A | 2207呎 (3房)
 -
 -
 (待售)</t>
@@ -4533,7 +4296,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>A | 1322呎 (4+房)
+          <t>A | 1322呎 (3房)
 -
 -
 (待售)</t>
@@ -4747,23 +4510,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>博峰 - 独立屋销控网格图</t>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>住宅大楼 - 西翼 销控网格图</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>总套数</t>
         </is>
@@ -4794,83 +4557,320 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="21" t="inlineStr">
-        <is>
-          <t>2 套</t>
-        </is>
-      </c>
-      <c r="B3" s="22" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="C3" s="23" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="D3" s="24" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="E3" s="25" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="F3" s="21" t="inlineStr">
-        <is>
-          <t>2 套</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>类型/位置</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>1号屋</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>2号屋</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>独立屋</t>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>楼层</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>A | 2217呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr"/>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>12</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>1号屋
-2623呎 (4+房)
-(待售)
-暂无价格
-暂无呎价</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>2号屋
-2621呎 (4+房)
-(待售)
-暂无价格
-暂无呎价</t>
+          <t>A | 2207呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr"/>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="58" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>

<commit_message>
feat(data): full update for 164 projects sales control & web dataset
</commit_message>
<xml_diff>
--- a/files/九龙-九龙塘-博峰.xlsx
+++ b/files/九龙-九龙塘-博峰.xlsx
@@ -8,9 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="销控汇总明细" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="独立屋销控表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="住宅大楼 - 东翼" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="住宅大楼 - 西翼" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="住宅大楼 - 东翼" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="住宅大楼 - 西翼" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="独立屋销控表" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4001,23 +4001,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>博峰 - 独立屋销控网格图</t>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>住宅大楼 - 东翼 销控网格图</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>总套数</t>
         </is>
@@ -4048,83 +4048,320 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="21" t="inlineStr">
-        <is>
-          <t>2 套</t>
-        </is>
-      </c>
-      <c r="B3" s="22" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="C3" s="23" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="D3" s="24" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="E3" s="25" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="F3" s="21" t="inlineStr">
-        <is>
-          <t>2 套</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>类型/位置</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>1号屋</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>2号屋</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>独立屋</t>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>楼层</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>A | 2217呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr"/>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>12</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>1号屋
-2623呎 (4+房)
-(待售)
-暂无价格
-暂无呎价</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>2号屋
-2621呎 (4+房)
-(待售)
-暂无价格
-暂无呎价</t>
+          <t>A | 2207呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr"/>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="58" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>A | 1322呎 (4+房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>B | 1089呎 (3房)
+-
+-
+(待售)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
@@ -4148,7 +4385,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>住宅大楼 - 东翼 销控网格图</t>
+          <t>住宅大楼 - 西翼 销控网格图</t>
         </is>
       </c>
     </row>
@@ -4257,7 +4494,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>A | 2207呎 (3房)
+          <t>A | 2207呎 (4+房)
 -
 -
 (待售)</t>
@@ -4296,7 +4533,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>A | 1322呎 (3房)
+          <t>A | 1322呎 (4+房)
 -
 -
 (待售)</t>
@@ -4510,23 +4747,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>住宅大楼 - 西翼 销控网格图</t>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>博峰 - 独立屋销控网格图</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>总套数</t>
         </is>
@@ -4557,320 +4794,83 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C3" s="14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E3" s="16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F3" s="17" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
-        <is>
-          <t>楼层</t>
-        </is>
-      </c>
-      <c r="B4" s="18" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C4" s="18" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>A | 2217呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C5" s="20" t="inlineStr"/>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>12</t>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>2 套</t>
+        </is>
+      </c>
+      <c r="B3" s="22" t="inlineStr">
+        <is>
+          <t>0 套</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>0 套</t>
+        </is>
+      </c>
+      <c r="D3" s="24" t="inlineStr">
+        <is>
+          <t>0 套</t>
+        </is>
+      </c>
+      <c r="E3" s="25" t="inlineStr">
+        <is>
+          <t>0 套</t>
+        </is>
+      </c>
+      <c r="F3" s="21" t="inlineStr">
+        <is>
+          <t>2 套</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>类型/位置</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>1号屋</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2号屋</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>独立屋</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>A | 2207呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C6" s="20" t="inlineStr"/>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C7" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="58" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="58" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="58" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B13" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C13" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="58" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="58" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C15" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="58" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>A | 1322呎 (4+房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="inlineStr">
-        <is>
-          <t>B | 1089呎 (3房)
--
--
-(待售)</t>
+          <t>1号屋
+2623呎 (4+房)
+(待售)
+暂无价格
+暂无呎价</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>2号屋
+2621呎 (4+房)
+(待售)
+暂无价格
+暂无呎价</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>